<commit_message>
fix: resolve blank black screen on Tasks, Routines, Goals, Projects, Calendar, Kanban, and Grid by adding loading state in App.jsx and passing timer controls
</commit_message>
<xml_diff>
--- a/Orbita_E2E_Test_Report.xlsx
+++ b/Orbita_E2E_Test_Report.xlsx
@@ -554,7 +554,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-20 07:33:03</t>
+          <t>2026-08-20 07:47:22</t>
         </is>
       </c>
     </row>
@@ -918,7 +918,7 @@
         </is>
       </c>
       <c r="F2" s="10" t="n">
-        <v>116.8</v>
+        <v>141.38</v>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
@@ -953,11 +953,11 @@
         </is>
       </c>
       <c r="F3" s="10" t="n">
-        <v>291.26</v>
+        <v>314.31</v>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Registered and logged in Member: e2e_tester_1787191327@orbita.com (ID: 6a86601ff95592b600062f91)</t>
+          <t>Registered and logged in Member: e2e_tester_1787192211@orbita.com (ID: 6a866393f95592b60006305c)</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
         </is>
       </c>
       <c r="F4" s="10" t="n">
-        <v>97.04000000000001</v>
+        <v>361.78</v>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
@@ -1023,11 +1023,11 @@
         </is>
       </c>
       <c r="F5" s="10" t="n">
-        <v>340.41</v>
+        <v>1016.2</v>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Created Task TSK-072 (Quadrant: Q2)</t>
+          <t>Created Task TSK-001 (Quadrant: Q2)</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1058,7 @@
         </is>
       </c>
       <c r="F6" s="10" t="n">
-        <v>181.1</v>
+        <v>424.64</v>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
@@ -1093,11 +1093,11 @@
         </is>
       </c>
       <c r="F7" s="10" t="n">
-        <v>290.12</v>
+        <v>283.71</v>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Task star toggled to True: 6a86601ff95592b600062f92</t>
+          <t>Task star toggled to True: 6a866394f95592b60006305d</t>
         </is>
       </c>
     </row>
@@ -1128,7 +1128,7 @@
         </is>
       </c>
       <c r="F8" s="10" t="n">
-        <v>257.8</v>
+        <v>273.03</v>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
@@ -1163,11 +1163,11 @@
         </is>
       </c>
       <c r="F9" s="10" t="n">
-        <v>361.29</v>
+        <v>337.9</v>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Created Daily Weekday Routine: RTN-015</t>
+          <t>Created Daily Weekday Routine: RTN-001</t>
         </is>
       </c>
     </row>
@@ -1198,11 +1198,11 @@
         </is>
       </c>
       <c r="F10" s="10" t="n">
-        <v>1519.31</v>
+        <v>334.33</v>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Created Weekly Multi-day Routine: RTN-016 (Days: Mon, Wed, Fri)</t>
+          <t>Created Weekly Multi-day Routine: RTN-002 (Days: Mon, Wed, Fri)</t>
         </is>
       </c>
     </row>
@@ -1233,11 +1233,11 @@
         </is>
       </c>
       <c r="F11" s="10" t="n">
-        <v>738.5599999999999</v>
+        <v>360.82</v>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Created Monthly Day 15 Routine: RTN-017</t>
+          <t>Created Monthly Day 15 Routine: RTN-003</t>
         </is>
       </c>
     </row>
@@ -1268,7 +1268,7 @@
         </is>
       </c>
       <c r="F12" s="10" t="n">
-        <v>18462.9</v>
+        <v>6565.49</v>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
@@ -1303,7 +1303,7 @@
         </is>
       </c>
       <c r="F13" s="10" t="n">
-        <v>13825.13</v>
+        <v>2907.6</v>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
@@ -1338,7 +1338,7 @@
         </is>
       </c>
       <c r="F14" s="10" t="n">
-        <v>547.99</v>
+        <v>1297.82</v>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
@@ -1373,11 +1373,11 @@
         </is>
       </c>
       <c r="F15" s="10" t="n">
-        <v>347.32</v>
+        <v>540.55</v>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Created Focus Goal GOL-010: Open hours tracking</t>
+          <t>Created Focus Goal GOL-001: Open hours tracking</t>
         </is>
       </c>
     </row>
@@ -1408,7 +1408,7 @@
         </is>
       </c>
       <c r="F16" s="10" t="n">
-        <v>3417.03</v>
+        <v>4493.76</v>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
@@ -1443,11 +1443,11 @@
         </is>
       </c>
       <c r="F17" s="10" t="n">
-        <v>689.87</v>
+        <v>148.27</v>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Timesheets endpoint verified: Found 4 logged sessions for member</t>
+          <t>Timesheets endpoint verified: Found 1 logged sessions for member</t>
         </is>
       </c>
     </row>
@@ -1478,11 +1478,11 @@
         </is>
       </c>
       <c r="F18" s="10" t="n">
-        <v>686.35</v>
+        <v>934.29</v>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>Created Project PRJ-003 with 2 Stages and 4 Sub-Tasks</t>
+          <t>Created Project PRJ-001 with 2 Stages and 4 Sub-Tasks</t>
         </is>
       </c>
     </row>
@@ -1513,7 +1513,7 @@
         </is>
       </c>
       <c r="F19" s="10" t="n">
-        <v>217.64</v>
+        <v>1083.44</v>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
         </is>
       </c>
       <c r="F20" s="10" t="n">
-        <v>283.24</v>
+        <v>774.0599999999999</v>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
@@ -1583,11 +1583,11 @@
         </is>
       </c>
       <c r="F21" s="10" t="n">
-        <v>2019.65</v>
+        <v>3593.86</v>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>Stage sub-task timer logged 1s directly</t>
+          <t>Stage sub-task timer logged 2s directly</t>
         </is>
       </c>
     </row>
@@ -1618,11 +1618,11 @@
         </is>
       </c>
       <c r="F22" s="10" t="n">
-        <v>6037.14</v>
+        <v>1965.91</v>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>Dashboard stats verified: Total=54, Completed=6, Hours=0.1h</t>
+          <t>Dashboard stats verified: Total=18, Completed=2, Hours=0h</t>
         </is>
       </c>
     </row>
@@ -1653,11 +1653,11 @@
         </is>
       </c>
       <c r="F23" s="10" t="n">
-        <v>5151.02</v>
+        <v>2097.28</v>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>Priority Matrix verified: Q1=0, Q2=48, Q3=0, Q4=0</t>
+          <t>Priority Matrix verified: Q1=0, Q2=16, Q3=0, Q4=0</t>
         </is>
       </c>
     </row>
@@ -1688,11 +1688,11 @@
         </is>
       </c>
       <c r="F24" s="10" t="n">
-        <v>208.2</v>
+        <v>195.51</v>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>Monthly Highlights verified: Month=August 2026, Score=105, Badges=2</t>
+          <t>Monthly Highlights verified: Month=August 2026, Score=35, Badges=1</t>
         </is>
       </c>
     </row>
@@ -1723,11 +1723,11 @@
         </is>
       </c>
       <c r="F25" s="10" t="n">
-        <v>84.98</v>
+        <v>88.48999999999999</v>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>Audit trail verified: 25 immutable event records (Latest: Task Focus Session Completed on PRJ-003-T1)</t>
+          <t>Audit trail verified: 9 immutable event records (Latest: Task Focus Session Completed on PRJ-001-T1)</t>
         </is>
       </c>
     </row>
@@ -1758,7 +1758,7 @@
         </is>
       </c>
       <c r="F26" s="10" t="n">
-        <v>338.62</v>
+        <v>368.06</v>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>

</xml_diff>